<commit_message>
updated handling of scientific committee subscribers
</commit_message>
<xml_diff>
--- a/_data/subscribers.xlsx
+++ b/_data/subscribers.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="234">
   <si>
     <t>Email</t>
   </si>
@@ -310,6 +310,27 @@
     <t>https://www.unimi.it/en/ugov/person/giulio-borghini</t>
   </si>
   <si>
+    <t>jacek.puziewicz@pm.me</t>
+  </si>
+  <si>
+    <t>Jacek</t>
+  </si>
+  <si>
+    <t>Puziewicz</t>
+  </si>
+  <si>
+    <t>University of Wroclaw</t>
+  </si>
+  <si>
+    <t>Wroclaw</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>petrology, mantle xenoliths,</t>
+  </si>
+  <si>
     <t>jfullea@ucm.es</t>
   </si>
   <si>
@@ -355,6 +376,27 @@
     <t>https://geodynamics.curtin.edu.au</t>
   </si>
   <si>
+    <t>maurizio.mazzucchelli@unimore.it</t>
+  </si>
+  <si>
+    <t>Maurizio</t>
+  </si>
+  <si>
+    <t>MAZZUCCHELLI</t>
+  </si>
+  <si>
+    <t>Dipartimento di Scienze Chimiche e Geologiche - Università di Modena e Reggio Emilia</t>
+  </si>
+  <si>
+    <t>Modena</t>
+  </si>
+  <si>
+    <t>petrology and geochemistry of mantle and lower crust</t>
+  </si>
+  <si>
+    <t>https://unimore.unifind.cineca.it/get/person/014255</t>
+  </si>
+  <si>
     <t>mavaras@uchile.cl</t>
   </si>
   <si>
@@ -400,6 +442,45 @@
     <t>Petrology</t>
   </si>
   <si>
+    <t>ndygert1@utk.edu</t>
+  </si>
+  <si>
+    <t>Nicholas</t>
+  </si>
+  <si>
+    <t>Dygert</t>
+  </si>
+  <si>
+    <t>University of Tennessee</t>
+  </si>
+  <si>
+    <t>Knoxville</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>petrology, geochemistry, experimental petrology, numerical modeling, rock deformation, planetary interiors</t>
+  </si>
+  <si>
+    <t>https://dygert.utk.edu</t>
+  </si>
+  <si>
+    <t>oelazar@carnegiescience.edu</t>
+  </si>
+  <si>
+    <t>Oded</t>
+  </si>
+  <si>
+    <t>Elazar</t>
+  </si>
+  <si>
+    <t>Carnegie science</t>
+  </si>
+  <si>
+    <t>Mantle geochemistry</t>
+  </si>
+  <si>
     <t>olivier.alard@anu.edu.au</t>
   </si>
   <si>
@@ -442,6 +523,18 @@
     <t>https://epss.hun-ren.hu/en/staff:patko.levente</t>
   </si>
   <si>
+    <t>patrizia.fumagalli@unimi.it</t>
+  </si>
+  <si>
+    <t>Patrizia</t>
+  </si>
+  <si>
+    <t>Fumagalli</t>
+  </si>
+  <si>
+    <t>Experimental Petrology</t>
+  </si>
+  <si>
     <t>romain.tilhac@umontpellier.fr</t>
   </si>
   <si>
@@ -457,9 +550,15 @@
     <t>Montpellier</t>
   </si>
   <si>
+    <t>petrology, geochemistry, isotope geochemistry, computational geochemistry</t>
+  </si>
+  <si>
     <t>https://romaintilhac.github.io</t>
   </si>
   <si>
+    <t>This application</t>
+  </si>
+  <si>
     <t>s.a.p.l.cloetingh@uu.nl</t>
   </si>
   <si>
@@ -502,6 +601,27 @@
     <t>https://www.esc.cam.ac.uk/people/sally-gibson</t>
   </si>
   <si>
+    <t>sarah.lambart@utah.edu</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Lambart</t>
+  </si>
+  <si>
+    <t>University of Utah</t>
+  </si>
+  <si>
+    <t>Salt Lake City</t>
+  </si>
+  <si>
+    <t>experimental petrology, high temperature geochemistry</t>
+  </si>
+  <si>
+    <t>http://sarahlambart.com/index.html</t>
+  </si>
+  <si>
     <t>stamatis.flemetakis@eaps.ethz.ch</t>
   </si>
   <si>
@@ -536,9 +656,6 @@
   </si>
   <si>
     <t>Newark</t>
-  </si>
-  <si>
-    <t>USA</t>
   </si>
   <si>
     <t>petrology, geochemistry, rheology, rock deformation</t>
@@ -942,7 +1059,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1376,7 +1493,7 @@
         <v>17</v>
       </c>
       <c r="J14" s="1">
-        <v>46311.540486111</v>
+        <v>46318.69931713</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1401,96 +1518,96 @@
       <c r="G15" t="s">
         <v>110</v>
       </c>
-      <c r="H15" t="s">
-        <v>111</v>
-      </c>
+      <c r="H15"/>
       <c r="I15" t="s">
         <v>17</v>
       </c>
       <c r="J15" s="1">
-        <v>46315.978761574</v>
+        <v>46311.540486111</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" t="s">
         <v>112</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>113</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>114</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>115</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>116</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>117</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>118</v>
       </c>
-      <c r="H16" t="s">
-        <v>119</v>
-      </c>
       <c r="I16" t="s">
         <v>17</v>
       </c>
       <c r="J16" s="1">
-        <v>46310.760185185</v>
+        <v>46315.978761574</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" t="s">
         <v>120</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>121</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>122</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>123</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17" t="s">
         <v>124</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H17" t="s">
         <v>125</v>
       </c>
-      <c r="G17" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17"/>
       <c r="I17" t="s">
         <v>17</v>
       </c>
       <c r="J17" s="1">
-        <v>46314.466284722</v>
+        <v>46318.700578704</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" t="s">
         <v>127</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>128</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>129</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>130</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>131</v>
-      </c>
-      <c r="F18" t="s">
-        <v>109</v>
       </c>
       <c r="G18" t="s">
         <v>132</v>
@@ -1502,7 +1619,7 @@
         <v>17</v>
       </c>
       <c r="J18" s="1">
-        <v>46314.903854167</v>
+        <v>46310.760185185</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1522,19 +1639,17 @@
         <v>138</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>139</v>
       </c>
       <c r="G19" t="s">
-        <v>139</v>
-      </c>
-      <c r="H19" t="s">
         <v>140</v>
       </c>
+      <c r="H19"/>
       <c r="I19" t="s">
         <v>17</v>
       </c>
       <c r="J19" s="1">
-        <v>46314.343009259</v>
+        <v>46314.466284722</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1554,71 +1669,69 @@
         <v>145</v>
       </c>
       <c r="F20" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G20" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="H20" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I20" t="s">
         <v>17</v>
       </c>
       <c r="J20" s="1">
-        <v>46310.518668981</v>
+        <v>46318.8078125</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="G21" t="s">
-        <v>151</v>
-      </c>
-      <c r="H21" t="s">
-        <v>152</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="H21"/>
       <c r="I21" t="s">
         <v>17</v>
       </c>
       <c r="J21" s="1">
-        <v>46318.630891204</v>
+        <v>46318.681574074</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F22" t="s">
-        <v>158</v>
+        <v>116</v>
       </c>
       <c r="G22" t="s">
         <v>159</v>
@@ -1630,7 +1743,7 @@
         <v>17</v>
       </c>
       <c r="J22" s="1">
-        <v>46318.376944444</v>
+        <v>46314.903854167</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1650,10 +1763,10 @@
         <v>165</v>
       </c>
       <c r="F23" t="s">
+        <v>74</v>
+      </c>
+      <c r="G23" t="s">
         <v>166</v>
-      </c>
-      <c r="G23" t="s">
-        <v>95</v>
       </c>
       <c r="H23" t="s">
         <v>167</v>
@@ -1662,7 +1775,7 @@
         <v>17</v>
       </c>
       <c r="J23" s="1">
-        <v>46317.462094907</v>
+        <v>46314.343009259</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1676,86 +1789,276 @@
         <v>170</v>
       </c>
       <c r="D24" t="s">
+        <v>51</v>
+      </c>
+      <c r="E24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" t="s">
         <v>171</v>
       </c>
-      <c r="E24" t="s">
-        <v>172</v>
-      </c>
-      <c r="F24" t="s">
-        <v>173</v>
-      </c>
-      <c r="G24" t="s">
-        <v>174</v>
-      </c>
-      <c r="H24" t="s">
-        <v>175</v>
-      </c>
+      <c r="H24"/>
       <c r="I24" t="s">
         <v>17</v>
       </c>
       <c r="J24" s="1">
-        <v>46312.520694444</v>
+        <v>46318.678402778</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" t="s">
+        <v>173</v>
+      </c>
+      <c r="C25" t="s">
+        <v>174</v>
+      </c>
+      <c r="D25" t="s">
+        <v>175</v>
+      </c>
+      <c r="E25" t="s">
         <v>176</v>
       </c>
-      <c r="B25" t="s">
+      <c r="F25" t="s">
+        <v>139</v>
+      </c>
+      <c r="G25" t="s">
         <v>177</v>
       </c>
-      <c r="C25" t="s">
+      <c r="H25" t="s">
         <v>178</v>
       </c>
-      <c r="D25" t="s">
+      <c r="I25" t="s">
         <v>179</v>
       </c>
-      <c r="E25" t="s">
-        <v>180</v>
-      </c>
-      <c r="F25" t="s">
-        <v>181</v>
-      </c>
-      <c r="G25" t="s">
-        <v>182</v>
-      </c>
-      <c r="H25"/>
-      <c r="I25" t="s">
-        <v>17</v>
-      </c>
       <c r="J25" s="1">
-        <v>46311.091967593</v>
+        <v>46310.518668981</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
+        <v>180</v>
+      </c>
+      <c r="B26" t="s">
+        <v>181</v>
+      </c>
+      <c r="C26" t="s">
+        <v>182</v>
+      </c>
+      <c r="D26" t="s">
         <v>183</v>
       </c>
-      <c r="B26" t="s">
+      <c r="E26" t="s">
+        <v>80</v>
+      </c>
+      <c r="F26" t="s">
+        <v>81</v>
+      </c>
+      <c r="G26" t="s">
         <v>184</v>
       </c>
-      <c r="C26" t="s">
+      <c r="H26" t="s">
         <v>185</v>
       </c>
-      <c r="D26" t="s">
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46318.630891204</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" t="s">
         <v>186</v>
       </c>
-      <c r="E26" t="s">
+      <c r="B27" t="s">
         <v>187</v>
       </c>
-      <c r="F26" t="s">
+      <c r="C27" t="s">
+        <v>188</v>
+      </c>
+      <c r="D27" t="s">
+        <v>189</v>
+      </c>
+      <c r="E27" t="s">
+        <v>190</v>
+      </c>
+      <c r="F27" t="s">
+        <v>191</v>
+      </c>
+      <c r="G27" t="s">
+        <v>192</v>
+      </c>
+      <c r="H27" t="s">
+        <v>193</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" s="1">
+        <v>46318.376944444</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" t="s">
+        <v>194</v>
+      </c>
+      <c r="B28" t="s">
+        <v>195</v>
+      </c>
+      <c r="C28" t="s">
+        <v>196</v>
+      </c>
+      <c r="D28" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" t="s">
+        <v>198</v>
+      </c>
+      <c r="F28" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" t="s">
+        <v>199</v>
+      </c>
+      <c r="H28" t="s">
+        <v>200</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" s="1">
+        <v>46318.691863426</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" t="s">
+        <v>201</v>
+      </c>
+      <c r="B29" t="s">
+        <v>202</v>
+      </c>
+      <c r="C29" t="s">
+        <v>203</v>
+      </c>
+      <c r="D29" t="s">
+        <v>204</v>
+      </c>
+      <c r="E29" t="s">
+        <v>205</v>
+      </c>
+      <c r="F29" t="s">
+        <v>206</v>
+      </c>
+      <c r="G29" t="s">
+        <v>95</v>
+      </c>
+      <c r="H29" t="s">
+        <v>207</v>
+      </c>
+      <c r="I29" t="s">
+        <v>17</v>
+      </c>
+      <c r="J29" s="1">
+        <v>46317.462094907</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" t="s">
+        <v>208</v>
+      </c>
+      <c r="B30" t="s">
+        <v>209</v>
+      </c>
+      <c r="C30" t="s">
+        <v>210</v>
+      </c>
+      <c r="D30" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" t="s">
+        <v>212</v>
+      </c>
+      <c r="F30" t="s">
+        <v>146</v>
+      </c>
+      <c r="G30" t="s">
+        <v>213</v>
+      </c>
+      <c r="H30" t="s">
+        <v>214</v>
+      </c>
+      <c r="I30" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" s="1">
+        <v>46312.520694444</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" t="s">
+        <v>215</v>
+      </c>
+      <c r="B31" t="s">
+        <v>216</v>
+      </c>
+      <c r="C31" t="s">
+        <v>217</v>
+      </c>
+      <c r="D31" t="s">
+        <v>218</v>
+      </c>
+      <c r="E31" t="s">
+        <v>219</v>
+      </c>
+      <c r="F31" t="s">
+        <v>220</v>
+      </c>
+      <c r="G31" t="s">
+        <v>221</v>
+      </c>
+      <c r="H31"/>
+      <c r="I31" t="s">
+        <v>17</v>
+      </c>
+      <c r="J31" s="1">
+        <v>46311.091967593</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" t="s">
+        <v>222</v>
+      </c>
+      <c r="B32" t="s">
+        <v>223</v>
+      </c>
+      <c r="C32" t="s">
+        <v>224</v>
+      </c>
+      <c r="D32" t="s">
+        <v>225</v>
+      </c>
+      <c r="E32" t="s">
+        <v>226</v>
+      </c>
+      <c r="F32" t="s">
         <v>68</v>
       </c>
-      <c r="G26" t="s">
-        <v>188</v>
-      </c>
-      <c r="H26" t="s">
-        <v>189</v>
-      </c>
-      <c r="I26" t="s">
-        <v>17</v>
-      </c>
-      <c r="J26" s="1">
+      <c r="G32" t="s">
+        <v>227</v>
+      </c>
+      <c r="H32" t="s">
+        <v>228</v>
+      </c>
+      <c r="I32" t="s">
+        <v>17</v>
+      </c>
+      <c r="J32" s="1">
         <v>46315.338506944</v>
       </c>
     </row>
@@ -1815,16 +2118,16 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="L1" t="s">
-        <v>191</v>
+        <v>230</v>
       </c>
       <c r="M1" t="s">
-        <v>192</v>
+        <v>231</v>
       </c>
       <c r="N1" t="s">
-        <v>193</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1883,7 +2186,7 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>194</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>